<commit_message>
fixing context retrieval during evaluation
</commit_message>
<xml_diff>
--- a/src/evaluation/data/ragas_results.xlsx
+++ b/src/evaluation/data/ragas_results.xlsx
@@ -507,12 +507,14 @@
         </is>
       </c>
       <c r="E2" t="n">
-        <v>0.7333333333333333</v>
+        <v>0.8</v>
       </c>
       <c r="F2" t="n">
         <v>0.8333333333333334</v>
       </c>
-      <c r="G2" t="inlineStr"/>
+      <c r="G2" t="n">
+        <v>0</v>
+      </c>
       <c r="H2" t="inlineStr">
         <is>
           <t>Studium-Übersicht</t>
@@ -555,7 +557,9 @@
       <c r="F3" t="n">
         <v>1</v>
       </c>
-      <c r="G3" t="inlineStr"/>
+      <c r="G3" t="n">
+        <v>0.4166666666458333</v>
+      </c>
       <c r="H3" t="inlineStr">
         <is>
           <t>Allgemein WiSo</t>
@@ -590,11 +594,15 @@
           <t>Für die regulären Studienprogramme fällt nur der halbjährliche Semesterbeitrag an, der bereits das Semesterticket für den öffentlichen Nahverkehr in ganz Nordrhein-Westfalen umfasst.</t>
         </is>
       </c>
-      <c r="E4" t="inlineStr"/>
+      <c r="E4" t="n">
+        <v>0.3333333333333333</v>
+      </c>
       <c r="F4" t="n">
         <v>0</v>
       </c>
-      <c r="G4" t="inlineStr"/>
+      <c r="G4" t="n">
+        <v>0</v>
+      </c>
       <c r="H4" t="inlineStr">
         <is>
           <t>Allgemein WiSo</t>
@@ -627,11 +635,15 @@
           <t>Mehrere DAX40-Vorstände haben an der UzK studiert, und laut dem Ranking des Magazins „Wirtschaftswoche“ werden WiSo-Absolvent:innen bei Einstellungen bevorzugt. Zudem erreicht die Fakultät im „Careers Rank“ des Financial Times Masters in Management Rankings eine Spitzenposition.</t>
         </is>
       </c>
-      <c r="E5" t="inlineStr"/>
+      <c r="E5" t="n">
+        <v>0.1666666666666667</v>
+      </c>
       <c r="F5" t="n">
         <v>0</v>
       </c>
-      <c r="G5" t="inlineStr"/>
+      <c r="G5" t="n">
+        <v>0.32499999998375</v>
+      </c>
       <c r="H5" t="inlineStr">
         <is>
           <t>Reputation/Ranking</t>
@@ -672,11 +684,15 @@
           <t>Die WiSo-Fakultät ist einziges deutsches Mitglied im CEMS-Netzwerk und bietet gemeinsam mit Partnern den Master in International Management (CEMS MIM) an. Viele Studienprogramme enthalten einen hohen Anteil englischsprachiger Module und nahezu alle Masterprogramme können vollständig auf Englisch studiert werden. Zudem bestehen Partnerschaften mit über 130 Hochschulen für Auslandssemester.</t>
         </is>
       </c>
-      <c r="E6" t="inlineStr"/>
+      <c r="E6" t="n">
+        <v>1</v>
+      </c>
       <c r="F6" t="n">
-        <v>1</v>
-      </c>
-      <c r="G6" t="inlineStr"/>
+        <v>0</v>
+      </c>
+      <c r="G6" t="n">
+        <v>0</v>
+      </c>
       <c r="H6" t="inlineStr">
         <is>
           <t>Internationalität</t>
@@ -715,12 +731,14 @@
         </is>
       </c>
       <c r="E7" t="n">
-        <v>0.8571428571428571</v>
+        <v>0.5</v>
       </c>
       <c r="F7" t="n">
         <v>1</v>
       </c>
-      <c r="G7" t="inlineStr"/>
+      <c r="G7" t="n">
+        <v>0</v>
+      </c>
       <c r="H7" t="inlineStr">
         <is>
           <t>Lehrinnovationen</t>
@@ -761,7 +779,9 @@
       <c r="F8" t="n">
         <v>1</v>
       </c>
-      <c r="G8" t="inlineStr"/>
+      <c r="G8" t="n">
+        <v>0</v>
+      </c>
       <c r="H8" t="inlineStr">
         <is>
           <t>Lehrinnovationen</t>
@@ -801,12 +821,14 @@
         </is>
       </c>
       <c r="E9" t="n">
-        <v>0.125</v>
+        <v>0.75</v>
       </c>
       <c r="F9" t="n">
         <v>0.5</v>
       </c>
-      <c r="G9" t="inlineStr"/>
+      <c r="G9" t="n">
+        <v>0</v>
+      </c>
       <c r="H9" t="inlineStr">
         <is>
           <t>Lehrinnovationen</t>
@@ -826,12 +848,18 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>["Kein Kontext gefunden"]</t>
+          <t>["mr\ne\nop Die Studierenden verteidigen ihre eigenständig und gemeinsam erarbeiteten\nKo\no Positionen und Problemlösungen. k\nh e …als aufgeklärt-emanzipierte, mündige und solidarische Persönlichkeit. c\niln\nö e\ntie\nk\ngn\nDie Studierenden entwickeln ein Verständnis für die Auswirkung von\ns\nr\nih gesellschaftlichen Entscheidungen unter Beachtung nachhaltiger, sozialer und/oder\ne ä\nP F ethischer Kriterien. 1", "8\n3 MODULBESCHREIBUNGEN UND MODULTABELLEN .................................... 9\n3.1 Modultabelle ........................................................................................................... 9\n3.2 Modulbeschreibungen ............................................................................................10\niv", "--- Page 99 ---\nMANAGEMENT, ECONOMICS AND SOCIAL SCIENCES. – BACHELOR OF SCIENCE\nGültig für Studierende der PO 2021 (Einschreibung ab WiSe 2021/22)\nSM Empirical Methods and Data Analysis\nKennnummer Workload LP Modulsprache Modulbeginn Moduldauer\n1314BSMDA1 180h 6 Deutsch und jedes 2. 1 Semester\nEnglisch Semester -\nWintersemester\n1 Lehrveranstaltungen Kontaktzeit Selbststudium LV-Sprache\nSelected Quantitative Methods 45h 135h Deutsch und\nEnglisch\n2 Inhalte des Moduls\nAusgewählte fortgeschrittene Methoden aus der Ökonometrie, zum Beispiel:\n• Asymptotische Eigenschaften des OLS-Schätzers\n• Allgemeine Schätzprinzipien\n• Heteroskedastie\n• Instrumentalvariablen\n• Einführung in die Zeitreihenanalyse (Einheitswurzeltests, GARCH)\n3 Lernziele des Moduls\nDie Studierenden... ... kennen und verstehen gängige Methoden aus dem Bereich Ökonometrie/Statistik. ... setzen Methoden aus dem Bereich Ökonometrie/Statistik in vorstrukturierten Kontexten\nlösungsorientiert ein. ... analysieren (aktuelle) Fragestellungen und Herausforderungen im Rahmen von vorstrukturierten\nKontexten. ... begründen und bewerten eigenständig erarbeitete Positionen. ... gestalten ihre Lern- und Arbeitsprozesse eigenständig. ... kennen und verstehen die relevanten Methoden und Theorien zu den zuvor unter \"Inhalte des\nModuls\" genannten Punkten.", "l!Die Wirtschafts- und Sozialwissenschaftliche Fakultät (WiSo-Fakultät) bietet ein breites Spektrum an englischsprachigen Masterstudiengängen mit exzellenter Lehre und Forschung, starken Unternehmens­kontakten und hervorragenden Karrierechancen.Wir laden Sie herzlich ein zumVirtuellen Infotag am 26. November 2025 um 17:00 Uhr, ein exklusives Event, das Ihnen einen direkten Einblick in Studium und Studierenden Leben an der WiSo-Fakultät gibt.Das erwartet Sie beim Event:Mehr über Köln, eine internationale, studierendenfreundliche StadtDie WiSo-Fakultät, eine Top-Fakultät mit 125 Jahren Erfahrung in der Ausbildung zukünftiger FührungskräfteMasterstudiengänge, darunter Deutschlands exklusiver CEMS Master in International Management sowie fünf Double-Degree-ProgrammeDie Services des WiSo Career Office und Ihre zukünftigen KarriereperspektivenBewerbungs- und ZulassungsverfahrenAngebote und Beratung für internationale StudierendeLernen Sie Vertreter:innen folgender Bereiche kennen:WiSo Student Service PointWiSo Career ServiceInternational OfficeZulassungsbüroProfessor:innen, aktuelle Studierende und AlumniDatum:26.", "Die Arbeiten in allen Paketen sind mit versorgungs- und patient:innenrelevanten Endpunkten verknüpft. Ergänzend werden die verschiedenen Perspektiven, sowohl der Betroffenen als auch der Leistungserbringenden, evaluiert.320px480px640px786px1024px1280px1440pxAuf Grundlage der Ergebnisse aus den verschiedenen Arbeitspaketen wird eine prozessorientierte Intervention zur Verbesserung der Koordination und Kooperation konzipiert, die zu einer Verbesserung der Versorgung von pädiatrischen Patient:innen mit (chronischen) Nierenerkrankungen führen soll.KontaktUoC Emerging Group HPDnetE-Mail:hpdnet-infouni-koeln.deProf. Dr. Ludwig Kuntz (Konsortialleitung)Universität zu Köln – Wirtschafts- und Sozialwissenschaftliche FakultätSeminar für ABWL und Management im GesundheitswesenTel.: +49 221 470- 5417Prof. Dr. Daniel WiesenUniversität zu Köln – Wirtschafts- und Sozialwissenschaftliche FakultätSeminar für ABWL und Management im GesundheitswesenTel.: +49 221 470- 89171Prof. Dr. Holger PfaffInstitut für Medizinsoziologie, Versorgungsforschung und Rehabilitationswissenschaft der Humanwissenschaftlichen Fakultät und der Medizinischen Fakultät der Universität zu Köln (IMVR)Zentrum für Versorgungsforschung Köln (ZVFK)Prof. Dr. Stephanie StockInstitut für Gesundheitsökonomie und Klinische Epidemiologie der Universität zu Köln (IGKE)Priv.-Doz. Dr."]</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>{"name": "university_knowledge_search", "parameters": {"query": "individualisierte E-Pr\u00fjfungen in E-PLUS"}}</t>
+          <t>Die individualisierten E-Prüfungen im Rahmen von E-PLUS bieten den Vorteil, dass die Studierenden ihre eigenen Lernprozesse individuell gestalten und ihre Lernziele erreichen können. Die Prüfungen sind nicht mehr auf eine einheitliche Note ausgerichtet, sondern ermöglichen es den Studenten, ihre eigene Leistung zu bewerten und zu verbessern.
+Durch die individualisierten E-Prüfungen können die Studierenden:
+* Ihre eigenen Lernziele setzen und erreichen
+* Ihre Lernprozesse individuell gestalten
+* Ihre Leistung selbstbewerten und verbessern
+* Mehr Autonomie und Selbstbestimmung in ihrem Lernprozess haben
+Die individualisierten E-Prüfungen ermöglichen es den Studenten, ihre eigenen Schwächen und Stärken zu erkennen und entsprechend anzupassen. Dies führt zu einer besseren Leistung und einem höheren Erfolg in der Ausbildung.</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -840,10 +868,10 @@
         </is>
       </c>
       <c r="E10" t="n">
-        <v>0</v>
+        <v>0.7777777777777778</v>
       </c>
       <c r="F10" t="n">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="G10" t="n">
         <v>0</v>
@@ -887,12 +915,14 @@
         </is>
       </c>
       <c r="E11" t="n">
-        <v>0.4166666666666667</v>
+        <v>1</v>
       </c>
       <c r="F11" t="n">
         <v>1</v>
       </c>
-      <c r="G11" t="inlineStr"/>
+      <c r="G11" t="n">
+        <v>0.8666666666377778</v>
+      </c>
       <c r="H11" t="inlineStr">
         <is>
           <t>Modulhandbuch/PO</t>
@@ -931,7 +961,9 @@
       <c r="F12" t="n">
         <v>1</v>
       </c>
-      <c r="G12" t="inlineStr"/>
+      <c r="G12" t="n">
+        <v>0.9999999999666667</v>
+      </c>
       <c r="H12" t="inlineStr">
         <is>
           <t>Modulhandbuch/PO</t>
@@ -971,12 +1003,14 @@
         </is>
       </c>
       <c r="E13" t="n">
-        <v>0.8333333333333334</v>
+        <v>0.125</v>
       </c>
       <c r="F13" t="n">
         <v>1</v>
       </c>
-      <c r="G13" t="inlineStr"/>
+      <c r="G13" t="n">
+        <v>0.5833333333041666</v>
+      </c>
       <c r="H13" t="inlineStr">
         <is>
           <t>Modulhandbuch/PO</t>
@@ -1017,7 +1051,9 @@
       <c r="F14" t="n">
         <v>1</v>
       </c>
-      <c r="G14" t="inlineStr"/>
+      <c r="G14" t="n">
+        <v>0.8333333332916666</v>
+      </c>
       <c r="H14" t="inlineStr">
         <is>
           <t>Modulhandbuch/PO</t>
@@ -1050,11 +1086,15 @@
           <t>Die Master-Dokumente gelten für Studierende der Prüfungsordnung 2021, die sich ab dem Wintersemester 2021/22 in einen der aufgeführten Masterstudiengänge eingeschrieben haben.</t>
         </is>
       </c>
-      <c r="E15" t="inlineStr"/>
+      <c r="E15" t="n">
+        <v>0.6666666666666666</v>
+      </c>
       <c r="F15" t="n">
         <v>1</v>
       </c>
-      <c r="G15" t="inlineStr"/>
+      <c r="G15" t="n">
+        <v>0.9999999999666667</v>
+      </c>
       <c r="H15" t="inlineStr">
         <is>
           <t>Modulhandbuch/PO</t>
@@ -1091,11 +1131,15 @@
           <t>Es werden u. a. Module für folgende Programme aufgeführt: M.Sc. International Management (CEMS MIM), mehrere Spezialisierungen im M.Sc. Business Administration (z. B. Finance, Marketing, Supply Chain Management), M.Sc. Business Analytics and Econometrics, M.Sc. Economics, M.Sc. Economic Research, M.Sc. Gesundheitsökonomie, M.Sc. Information Systems, Master-Programme in Politikwissenschaft sowie zwei Soziologie-Master und Wirtschaftspädagogik.</t>
         </is>
       </c>
-      <c r="E16" t="inlineStr"/>
+      <c r="E16" t="n">
+        <v>0.2</v>
+      </c>
       <c r="F16" t="n">
         <v>1</v>
       </c>
-      <c r="G16" t="inlineStr"/>
+      <c r="G16" t="n">
+        <v>0</v>
+      </c>
       <c r="H16" t="inlineStr">
         <is>
           <t>Modulhandbuch/PO</t>
@@ -1133,11 +1177,15 @@
           <t>Die gemeinsame Prüfungsordnung der WiSo-Masterstudiengänge sowie eine zusätzliche Masterprüfungsordnung sind über den verlinkten Download-Bereich des Prüfungsamtes auf folgender Seite abrufbar: https://wiso.uni-koeln.de/de/studium/modulhandbuecher-und-pruefungsordnungen/master-po-2021</t>
         </is>
       </c>
-      <c r="E17" t="inlineStr"/>
+      <c r="E17" t="n">
+        <v>0</v>
+      </c>
       <c r="F17" t="n">
         <v>1</v>
       </c>
-      <c r="G17" t="inlineStr"/>
+      <c r="G17" t="n">
+        <v>0</v>
+      </c>
       <c r="H17" t="inlineStr">
         <is>
           <t>Modulhandbuch/PO</t>
@@ -1184,7 +1232,9 @@
       <c r="F18" t="n">
         <v>0</v>
       </c>
-      <c r="G18" t="inlineStr"/>
+      <c r="G18" t="n">
+        <v>0</v>
+      </c>
       <c r="H18" t="inlineStr">
         <is>
           <t>Bachelor-Studium</t>
@@ -1227,7 +1277,9 @@
       <c r="F19" t="n">
         <v>1</v>
       </c>
-      <c r="G19" t="inlineStr"/>
+      <c r="G19" t="n">
+        <v>0.3333333333</v>
+      </c>
       <c r="H19" t="inlineStr">
         <is>
           <t>Bachelor-Studium</t>
@@ -1247,15 +1299,13 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>["Kein Kontext gefunden"]</t>
+          <t>["--- Page 24 ---\nMANAGEMENT, ECONOMICS AND SOCIAL SCIENCES. – BACHELOR OF SCIENCE\nGültig für Studierende der PO 2021 (Einschreibung ab WiSe 2021/22)\n3.5 Bachelorarbeit\nDie Bachelorarbeit umfasst 12 LP und wird studienbegleitend zu Ende des Studiums erstellt. Die Anmeldung von Abschlussarbeiten erfolgt bei den verschiedenen Lehrstühlen nur in der\nersten Zulassungsphase in KLIPS. Mit ihr wird gezeigt, dass ein thematisch begrenztes\nProblem aus dem Gegenstandsbereich des Studiengangs mit den erforderlichen Methoden in\neinem festgelegten Zeitraum wissenschaftlich bearbeitet und reflektiert werden kann. Das\nThema der Bachelorarbeit kann aus dem gesamten Gegenstandsbereich des Studiums\nentnommen werden. Die Bachelorarbeit kann auch in Form einer Gruppenarbeit geschrieben\nwerden, wenn der Beitrag jedes/jeder einzelnen Geprüften deutlich unterscheidbar und\nbewertbar ist. Die Zuordnung des individuellen Beitrags erfolgt aufgrund von objektiven\nKriterien, die eine eindeutige Abgrenzung ermöglichen, bspw. durch die Angabe von\nAbschnitten, Seitenzahlen oder inhaltlichen Schwerpunkten. Der insgesamt für eine\nGruppenarbeit erforderliche Arbeitsaufwand muss über die Anforderungen an eine\nEinzelaufgabe angemessen hinausgehen. Nach Schwierigkeitsgrad und Inhalt ist eine\nGruppenarbeit für jedes einzelne Gruppenmitglied so zu bemessen, dass sie den\nAnforderungen an eine individuelle und selbstständige Prüfungsleistung entspricht.", "Semester besucht werden. Die Bachelorarbeit – soweit diese zum Studienbereich der beruflichen Fachrichtung Wirt-\nschaftswissenschaften angefertigt wird – sollte zu den fachdidaktisch ausgerichteten Schwer-\npunktmodulen angefertigt werden. 2", "in einen persönlichen Studienplan integriert werden. Achten Sie bei der\nindividuellen Planung auf mögliche Überschneidungen von Lehrveranstaltungen. Bei weiteren\nFragen hilft der WiSo Student Service Point gerne weiter. Der nachfolgende\nMusterstudienplan zeigt den gewöhnlichen Studienverlauf auf.\n7\n\n--- Page 12 ---\nMANAGEMENT, ECONOMICS AND SOCIAL SCIENCES. – BACHELOR OF SCIENCE\nGültig für Studierende der PO 2021 (Einschreibung ab WiSe 2021/22)\nB.Sc", "l!Die Wirtschafts- und Sozialwissenschaftliche Fakultät (WiSo-Fakultät) bietet ein breites Spektrum an englischsprachigen Masterstudiengängen mit exzellenter Lehre und Forschung, starken Unternehmens­kontakten und hervorragenden Karrierechancen.Wir laden Sie herzlich ein zumVirtuellen Infotag am 26. November 2025 um 17:00 Uhr, ein exklusives Event, das Ihnen einen direkten Einblick in Studium und Studierenden Leben an der WiSo-Fakultät gibt.Das erwartet Sie beim Event:Mehr über Köln, eine internationale, studierendenfreundliche StadtDie WiSo-Fakultät, eine Top-Fakultät mit 125 Jahren Erfahrung in der Ausbildung zukünftiger FührungskräfteMasterstudiengänge, darunter Deutschlands exklusiver CEMS Master in International Management sowie fünf Double-Degree-ProgrammeDie Services des WiSo Career Office und Ihre zukünftigen KarriereperspektivenBewerbungs- und ZulassungsverfahrenAngebote und Beratung für internationale StudierendeLernen Sie Vertreter:innen folgender Bereiche kennen:WiSo Student Service PointWiSo Career ServiceInternational OfficeZulassungsbüroProfessor:innen, aktuelle Studierende und AlumniDatum:26.", "Mit dem gezielten Auf- und Ausbau von strukturierter Doktorand*innenausbildung wurden von der Universität zu Köln exzellente Rahmenbedingungen für Promovierende geschaffen. DieCologne Graduate School in Management, Economics and Social Sciences(CGS) stellt das Dach für alle Promovierenden der WiSo-Fakultät dar. Über zahlreiche Vernetzungs- und Weiterbildungsangebote für PostDocs wird die wissenschaftliche Weiterentwicklung gezielt unterstützt. \"My idea is to face the world with its challenges and find ways to have a positive impact\" Lena,Studentin imB.Sc. Management, Economics and Social Sciences Mit der Gründung des universitätsweitenAlbertus Magnus Center(AMC) im Rahmen desZukunftskonzeptswerden die verschiedenen Strukturen zusammengeführt. Promotion an der WiSo-Fakultät Albertus Magnus Center Junior Faculty Club Postdoc Career Program Personalentwicklung Wissenschaft Transferunterstützung Female Career Center (FCC) Cornelia Harte Mentoring Erste Generation Promotion Mentoring+ Gender Mentoring-Agentur Mentoring Program for International Female Scholars Mentoring Program for Scholars at Risk zum Seitenanfang"]</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Laut den Suchergebnissen ist der Standort Köln für Studierende attraktiv aufgrund seiner Vielfalt an Kursen, seiner Nähe zu Unternehmen und seiner Möglichkeiten zur Praxisorientierung. Außerdem bietet die Universität Köln ein breites Spektrum an Studiengängen an, darunter auch einige, die stark praxisorientiert sind.
-Zusätzlich bieten viele der genannten Quellen Vorteile des Studierens in den Niederlanden oder in Nordrhein-Westfalen an, wie zum Beispiel eine gute Qualität der Hochschulen oder Möglichkeiten zur Finanzierung des Studiums.
-Quelle: DuckDuckGo-Suchergebnisse für 'Köln als Studienstandort, Vorteile für Studenten'
-URL: https://duckduckgo.com/</t>
+          <t>Der Standort Köln ist laut Bachelorseite für Studierende attraktiv, da die Universität zu Köln eine Top-Fakultät mit 125 Jahren Erfahrung in der Ausbildung zukünftiger Führungskräfte bietet. Die WiSo-Fakultät bietet ein breites Spektrum an englischsprachigen Masterstudiengängen mit exzellenter Lehre und Forschung, starken Unternehmenskontakten und hervorragenden Karrierechancen. Die Stadt Köln ist internationale, studierendenfreundlich und bietet eine Vielzahl von Möglichkeiten für das persönliche Leben der Studierenden.
+URL: https://wiso.uni-koeln.de/de/studium/bachelor-management-economics-social-sciences/</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
@@ -1264,10 +1314,10 @@
         </is>
       </c>
       <c r="E20" t="n">
-        <v>0.25</v>
+        <v>0.75</v>
       </c>
       <c r="F20" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G20" t="n">
         <v>0</v>
@@ -1296,9 +1346,10 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Es tut mir leid, aber ich konnte keine Informationen über "Chat with Paco" finden. Es ist möglich, dass es sich um ein spezielles Angebot handelt, das nicht öffentlich verfügbar ist oder kein bekanntes Konzept ist.
-Wenn du mehr wissen möchtest, kannst du versuchen, eine Suche im Internet durchzuführen, um weitere Informationen zu finden. Ich kann dir gerne dabei helfen, wenn du ein bestimmtes Thema suche.
-Ich hoffe, das hilft! Wenn du noch Fragen hast, stehe ich gerne zur Verfügung.</t>
+          <t>Entschuldigung, ich habe das Ergebnis nicht verstanden.
+"Chat with Paco" ist ein Angebot für persönliche und intelligente Gespräche mit einem Charakter namens Paco. Es bietet eine Möglichkeit, mit einem AI-Chatbot zu sprechen, der auf individuellen Bedürfnissen basiert. Paco kann als Amable, verantwortungsvoll und freundlich beschrieben werden.
+Es gibt verschiedene Anbieter von "Chat with Paco", wie z.B. Polybuzz.ai, character.ai, Talkie-AI und Joyland.ai. Jeder bietet eine eigene Plattform für die Interaktion mit Paco.
+Wenn du also nach einem Chatbot suchst, der dir individuelle Antworten und Unterhaltungen bieten kann, könntest du "Chat with Paco" in Erwägung ziehen.</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
@@ -1357,12 +1408,14 @@
         </is>
       </c>
       <c r="E22" t="n">
-        <v>0.5555555555555556</v>
+        <v>0.1111111111111111</v>
       </c>
       <c r="F22" t="n">
         <v>1</v>
       </c>
-      <c r="G22" t="inlineStr"/>
+      <c r="G22" t="n">
+        <v>0.8333333332916666</v>
+      </c>
       <c r="H22" t="inlineStr">
         <is>
           <t>Verbundstudiengänge</t>
@@ -1396,11 +1449,15 @@
           <t>Im B.Sc. Geographie müssen zwei Nebenfächer gewählt werden, wobei auch BWL, VWL oder Sozialwissenschaften der WiSo-Fakultät möglich sind. Für diese drei Nebenfächer ist jedoch ein Motivationsschreiben erforderlich, das an die im Geographie-Hinweis genannte Kontaktperson gerichtet werden muss – nicht an den WiSo Student Service Point.</t>
         </is>
       </c>
-      <c r="E23" t="inlineStr"/>
+      <c r="E23" t="n">
+        <v>0.3333333333333333</v>
+      </c>
       <c r="F23" t="n">
         <v>0.5</v>
       </c>
-      <c r="G23" t="inlineStr"/>
+      <c r="G23" t="n">
+        <v>0</v>
+      </c>
       <c r="H23" t="inlineStr">
         <is>
           <t>Verbundstudiengänge</t>
@@ -1433,11 +1490,15 @@
           <t>Für das Wintersemester endet die Bewerbungsfrist regulär am 15. Juli, für das Sommersemester am 15. Januar. Ein Studienstart im Sommersemester ist zusätzlich nur in den Bachelorstudiengängen Betriebswirtschaftslehre und Volkswirtschaftslehre möglich.</t>
         </is>
       </c>
-      <c r="E24" t="inlineStr"/>
+      <c r="E24" t="n">
+        <v>0.3333333333333333</v>
+      </c>
       <c r="F24" t="n">
         <v>0</v>
       </c>
-      <c r="G24" t="inlineStr"/>
+      <c r="G24" t="n">
+        <v>0</v>
+      </c>
       <c r="H24" t="inlineStr">
         <is>
           <t>Bewerbung Bachelor</t>
@@ -1472,11 +1533,15 @@
           <t>Internationale Studieninteressierte sollen sich vor der Bewerbung beim International Office der Universität zu Köln über das jeweilige Bewerbungsverfahren informieren; der entsprechende Link ist auf der Bachelor-Bewerbungsseite hinterlegt.</t>
         </is>
       </c>
-      <c r="E25" t="inlineStr"/>
+      <c r="E25" t="n">
+        <v>1</v>
+      </c>
       <c r="F25" t="n">
         <v>0.5</v>
       </c>
-      <c r="G25" t="inlineStr"/>
+      <c r="G25" t="n">
+        <v>0</v>
+      </c>
       <c r="H25" t="inlineStr">
         <is>
           <t>Bewerbung Bachelor</t>
@@ -1515,7 +1580,9 @@
       <c r="F26" t="n">
         <v>1</v>
       </c>
-      <c r="G26" t="inlineStr"/>
+      <c r="G26" t="n">
+        <v>0</v>
+      </c>
       <c r="H26" t="inlineStr">
         <is>
           <t>Bewerbung Bachelor</t>
@@ -1553,11 +1620,15 @@
           <t>Die Seite stellt klar, dass beruflich Qualifizierte ohne Abitur unter bestimmten Voraussetzungen studieren können; je nach beruflicher Vorbildung unterscheiden sich die Zugangswege. Konkrete Informationen zu Bewerbergruppen und Verfahren sind über die verlinkten Seiten der zentralen Verwaltung abrufbar.</t>
         </is>
       </c>
-      <c r="E27" t="inlineStr"/>
+      <c r="E27" t="n">
+        <v>0.8333333333333334</v>
+      </c>
       <c r="F27" t="n">
         <v>0.3333333333333333</v>
       </c>
-      <c r="G27" t="inlineStr"/>
+      <c r="G27" t="n">
+        <v>0.5833333333041666</v>
+      </c>
       <c r="H27" t="inlineStr">
         <is>
           <t>Bewerbung Bachelor</t>
@@ -1600,7 +1671,9 @@
       <c r="F28" t="n">
         <v>0.5</v>
       </c>
-      <c r="G28" t="inlineStr"/>
+      <c r="G28" t="n">
+        <v>0.3666666666483334</v>
+      </c>
       <c r="H28" t="inlineStr">
         <is>
           <t>Services/Info</t>
@@ -1640,12 +1713,14 @@
         </is>
       </c>
       <c r="E29" t="n">
-        <v>0.5</v>
+        <v>0.75</v>
       </c>
       <c r="F29" t="n">
         <v>1</v>
       </c>
-      <c r="G29" t="inlineStr"/>
+      <c r="G29" t="n">
+        <v>0.49999999995</v>
+      </c>
       <c r="H29" t="inlineStr">
         <is>
           <t>Bewerbung Master</t>
@@ -1688,7 +1763,9 @@
       <c r="F30" t="n">
         <v>1</v>
       </c>
-      <c r="G30" t="inlineStr"/>
+      <c r="G30" t="n">
+        <v>0</v>
+      </c>
       <c r="H30" t="inlineStr">
         <is>
           <t>Bewerbung Master</t>
@@ -1734,7 +1811,9 @@
       <c r="F31" t="n">
         <v>1</v>
       </c>
-      <c r="G31" t="inlineStr"/>
+      <c r="G31" t="n">
+        <v>0.9999999999666667</v>
+      </c>
       <c r="H31" t="inlineStr">
         <is>
           <t>Bewerbung Master</t>
@@ -1771,11 +1850,15 @@
           <t>Am Ende der Master-Bewerbungsseite sind die einzelnen Masterstudiengänge jeweils mit eigenen Informationsseiten verlinkt, darunter auch eine Seite speziell zum Master Information Systems.</t>
         </is>
       </c>
-      <c r="E32" t="inlineStr"/>
+      <c r="E32" t="n">
+        <v>1</v>
+      </c>
       <c r="F32" t="n">
         <v>1</v>
       </c>
-      <c r="G32" t="inlineStr"/>
+      <c r="G32" t="n">
+        <v>0.9999999999</v>
+      </c>
       <c r="H32" t="inlineStr">
         <is>
           <t>Bewerbung Master</t>
@@ -1816,11 +1899,15 @@
           <t>Der Master Information Systems schließt mit einem Master of Science ab, dauert vier Semester in Vollzeit und umfasst 120 ECTS. Die Unterrichtssprache ist überwiegend Englisch, einzelne Kurse werden auf Deutsch angeboten. Es bestehen optionale internationale Elemente wie Auslandssemester und Summer Schools.</t>
         </is>
       </c>
-      <c r="E33" t="inlineStr"/>
+      <c r="E33" t="n">
+        <v>0.1666666666666667</v>
+      </c>
       <c r="F33" t="n">
         <v>0.75</v>
       </c>
-      <c r="G33" t="inlineStr"/>
+      <c r="G33" t="n">
+        <v>0</v>
+      </c>
       <c r="H33" t="inlineStr">
         <is>
           <t>MIS-Überblick</t>
@@ -1857,11 +1944,15 @@
           <t>Das Programm behandelt die interdisziplinäre Disziplin der Wirtschaftsinformatik an der Schnittstelle von Betriebswirtschaftslehre und Informatik. Im Fokus stehen Konzeption, Entwicklung und Anwendung von Informationssystemen in Unternehmen, Verwaltung und zunehmend im privaten Bereich.</t>
         </is>
       </c>
-      <c r="E34" t="inlineStr"/>
+      <c r="E34" t="n">
+        <v>0.5</v>
+      </c>
       <c r="F34" t="n">
         <v>1</v>
       </c>
-      <c r="G34" t="inlineStr"/>
+      <c r="G34" t="n">
+        <v>0</v>
+      </c>
       <c r="H34" t="inlineStr">
         <is>
           <t>MIS-Inhalt</t>
@@ -1899,12 +1990,14 @@
         </is>
       </c>
       <c r="E35" t="n">
-        <v>0.6</v>
+        <v>0.4</v>
       </c>
       <c r="F35" t="n">
         <v>1</v>
       </c>
-      <c r="G35" t="inlineStr"/>
+      <c r="G35" t="n">
+        <v>0</v>
+      </c>
       <c r="H35" t="inlineStr">
         <is>
           <t>MIS-Bewerbung</t>
@@ -1948,11 +2041,15 @@
           <t>Genannt werden u. a. theoretische und methodische Grundlagen für Themen wie Data Science, digitale Transformation und Innovation, Prozesse und Geschäftsmodelle sowie Lösungen für eine nachhaltige Gesellschaft. Außerdem wird die Ausbildung im interdisziplinären Bereich der Wirtschaftsinformatik betont, die die gefragte Fähigkeit vermittelt, BWL und Informatik zu verbinden.</t>
         </is>
       </c>
-      <c r="E36" t="inlineStr"/>
+      <c r="E36" t="n">
+        <v>0</v>
+      </c>
       <c r="F36" t="n">
         <v>1</v>
       </c>
-      <c r="G36" t="inlineStr"/>
+      <c r="G36" t="n">
+        <v>0</v>
+      </c>
       <c r="H36" t="inlineStr">
         <is>
           <t>MIS-Inhalt</t>
@@ -1997,11 +2094,15 @@
           <t>Geeignet ist das Programm für Bewerber:innen mit Bachelorabschluss in Informatik, Wirtschaftsinformatik, Wirtschaftswissenschaften, Betriebswirtschaft oder verwandten Fächern, die über technische Fähigkeiten in Mathematik/Statistik und Informatik (insbesondere Programmierung) verfügen, gerne in internationalen, interkulturellen Teams arbeiten und bereit sind, den nächsten Karriereschritt als breit aufgestellte Wirtschaftsinformatiker:innen zu gehen.</t>
         </is>
       </c>
-      <c r="E37" t="inlineStr"/>
+      <c r="E37" t="n">
+        <v>0.8181818181818182</v>
+      </c>
       <c r="F37" t="n">
         <v>0.5</v>
       </c>
-      <c r="G37" t="inlineStr"/>
+      <c r="G37" t="n">
+        <v>0.9999999999</v>
+      </c>
       <c r="H37" t="inlineStr">
         <is>
           <t>MIS-Zielgruppe</t>
@@ -2039,11 +2140,15 @@
           <t>Der Studiengang wird vom Kölner Institut für Wirtschaftsinformatik (CIIS) ausgerichtet. Laut Beschreibung zählen mehrere Professoren des CIIS im WirtschaftsWoche-Ranking zu den Top 5 % der Wirtschaftsforscher:innen im deutschsprachigen Raum, und das CIIS belegt im AIS-Ranking 2022 Spitzenpositionen (Platz 1 in Deutschland, Top 10 in Europa, Top 100 weltweit).</t>
         </is>
       </c>
-      <c r="E38" t="inlineStr"/>
+      <c r="E38" t="n">
+        <v>0.8</v>
+      </c>
       <c r="F38" t="n">
         <v>0.3333333333333333</v>
       </c>
-      <c r="G38" t="inlineStr"/>
+      <c r="G38" t="n">
+        <v>0.9999999999</v>
+      </c>
       <c r="H38" t="inlineStr">
         <is>
           <t>MIS-Ranking</t>
@@ -2077,11 +2182,15 @@
           <t>Die Fakultät hebt ihre langjährige Erfahrung in der Zusammenarbeit mit Unternehmen und Gastdozent:innen aus verschiedenen Berufsfeldern hervor. Diese bringen aktuelle Branchenerfahrung in das Programm ein, sodass Inhalte Praxis und Theorie eng verbinden und reale Entwicklungen widerspiegeln.</t>
         </is>
       </c>
-      <c r="E39" t="inlineStr"/>
+      <c r="E39" t="n">
+        <v>0.6666666666666666</v>
+      </c>
       <c r="F39" t="n">
         <v>1</v>
       </c>
-      <c r="G39" t="inlineStr"/>
+      <c r="G39" t="n">
+        <v>0</v>
+      </c>
       <c r="H39" t="inlineStr">
         <is>
           <t>Praxisbezug</t>
@@ -2124,7 +2233,9 @@
       <c r="F40" t="n">
         <v>1</v>
       </c>
-      <c r="G40" t="inlineStr"/>
+      <c r="G40" t="n">
+        <v>0.699999999965</v>
+      </c>
       <c r="H40" t="inlineStr">
         <is>
           <t>Beratung</t>

</xml_diff>